<commit_message>
insert spline interpolation, create crqa folder, replace median with mean
</commit_message>
<xml_diff>
--- a/Best ch pipeline/improved_best_channels_stat.xlsx
+++ b/Best ch pipeline/improved_best_channels_stat.xlsx
@@ -662,19 +662,19 @@
         <v>126453</v>
       </c>
       <c r="E7" t="n">
-        <v>600</v>
+        <v>587</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>46.90922428222573</v>
+        <v>54.6846528203046</v>
       </c>
       <c r="H7" t="n">
-        <v>210.2716666666667</v>
+        <v>214.9284497444634</v>
       </c>
       <c r="I7" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8">
@@ -1256,16 +1256,16 @@
         <v>149903</v>
       </c>
       <c r="E25" t="n">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="F25" t="n">
         <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>38.29382421846555</v>
+        <v>38.96217293991534</v>
       </c>
       <c r="H25" t="n">
-        <v>214.3810888252149</v>
+        <v>214.6886657101865</v>
       </c>
       <c r="I25" t="n">
         <v>208</v>
@@ -1619,19 +1619,19 @@
         <v>150053</v>
       </c>
       <c r="E36" t="n">
-        <v>569</v>
+        <v>524</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>637.0658658683889</v>
+        <v>665.2150524470057</v>
       </c>
       <c r="H36" t="n">
-        <v>263.1318101933216</v>
+        <v>285.7290076335878</v>
       </c>
       <c r="I36" t="n">
-        <v>234</v>
+        <v>239.5</v>
       </c>
     </row>
     <row r="37">
@@ -1652,19 +1652,19 @@
         <v>147583</v>
       </c>
       <c r="E37" t="n">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="F37" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G37" t="n">
-        <v>1168.369872788458</v>
+        <v>1215.649782895623</v>
       </c>
       <c r="H37" t="n">
-        <v>720.1127450980392</v>
+        <v>769.1256544502618</v>
       </c>
       <c r="I37" t="n">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="38">
@@ -1685,19 +1685,19 @@
         <v>150146</v>
       </c>
       <c r="E38" t="n">
-        <v>628</v>
+        <v>594</v>
       </c>
       <c r="F38" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G38" t="n">
-        <v>154.3570465411999</v>
+        <v>165.3760084809848</v>
       </c>
       <c r="H38" t="n">
-        <v>238.5764331210191</v>
+        <v>252.2323232323232</v>
       </c>
       <c r="I38" t="n">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="39">
@@ -2279,19 +2279,19 @@
         <v>150333</v>
       </c>
       <c r="E56" t="n">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="F56" t="n">
         <v>4</v>
       </c>
       <c r="G56" t="n">
-        <v>855.9063164464903</v>
+        <v>857.4049380320445</v>
       </c>
       <c r="H56" t="n">
-        <v>255.2874149659864</v>
+        <v>256.1587030716723</v>
       </c>
       <c r="I56" t="n">
-        <v>212</v>
+        <v>212.5</v>
       </c>
     </row>
     <row r="57">
@@ -2345,19 +2345,19 @@
         <v>150089</v>
       </c>
       <c r="E58" t="n">
-        <v>657</v>
+        <v>642</v>
       </c>
       <c r="F58" t="n">
         <v>3</v>
       </c>
       <c r="G58" t="n">
-        <v>68.51502869115996</v>
+        <v>73.90515916143966</v>
       </c>
       <c r="H58" t="n">
-        <v>227.9573820395738</v>
+        <v>233.2834890965732</v>
       </c>
       <c r="I58" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="59">
@@ -2378,16 +2378,16 @@
         <v>150138</v>
       </c>
       <c r="E59" t="n">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F59" t="n">
         <v>2</v>
       </c>
       <c r="G59" t="n">
-        <v>3248.825742812279</v>
+        <v>3252.913349193057</v>
       </c>
       <c r="H59" t="n">
-        <v>377.3853904282116</v>
+        <v>378.3383838383838</v>
       </c>
       <c r="I59" t="n">
         <v>213</v>
@@ -2642,19 +2642,19 @@
         <v>59893</v>
       </c>
       <c r="E67" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F67" t="n">
         <v>36</v>
       </c>
       <c r="G67" t="n">
-        <v>469.3268835771313</v>
+        <v>472.7954082549981</v>
       </c>
       <c r="H67" t="n">
-        <v>593.3163265306123</v>
+        <v>599.4329896907217</v>
       </c>
       <c r="I67" t="n">
-        <v>391</v>
+        <v>409</v>
       </c>
     </row>
     <row r="68">
@@ -2708,16 +2708,16 @@
         <v>110120</v>
       </c>
       <c r="E69" t="n">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="F69" t="n">
         <v>3</v>
       </c>
       <c r="G69" t="n">
-        <v>75.877475373615</v>
+        <v>84.10424543944512</v>
       </c>
       <c r="H69" t="n">
-        <v>250.1480637813212</v>
+        <v>251.2929061784897</v>
       </c>
       <c r="I69" t="n">
         <v>240</v>
@@ -3033,19 +3033,19 @@
         <v>150073</v>
       </c>
       <c r="E3" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G3" t="n">
-        <v>1266.670528125103</v>
+        <v>1270.802678657989</v>
       </c>
       <c r="H3" t="n">
-        <v>924.0083333333333</v>
+        <v>931.7731092436975</v>
       </c>
       <c r="I3" t="n">
-        <v>423.5</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4">
@@ -3324,25 +3324,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>149.99</v>
+        <v>149.707</v>
       </c>
       <c r="D12" t="n">
-        <v>149990</v>
+        <v>149707</v>
       </c>
       <c r="E12" t="n">
-        <v>474</v>
+        <v>451</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>82.00392047790697</v>
+        <v>103.8239033513958</v>
       </c>
       <c r="H12" t="n">
-        <v>315.632911392405</v>
+        <v>331.1019955654102</v>
       </c>
       <c r="I12" t="n">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="13">
@@ -3396,19 +3396,19 @@
         <v>149498</v>
       </c>
       <c r="E14" t="n">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F14" t="n">
         <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>161.95345404552</v>
+        <v>160.6564431564435</v>
       </c>
       <c r="H14" t="n">
-        <v>455.7675840978594</v>
+        <v>454.3780487804878</v>
       </c>
       <c r="I14" t="n">
-        <v>485</v>
+        <v>484.5</v>
       </c>
     </row>
     <row r="15">
@@ -3429,19 +3429,19 @@
         <v>98601</v>
       </c>
       <c r="E15" t="n">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G15" t="n">
-        <v>234.4780014841328</v>
+        <v>239.8865782982235</v>
       </c>
       <c r="H15" t="n">
-        <v>430.4096916299559</v>
+        <v>436.1741071428572</v>
       </c>
       <c r="I15" t="n">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="16">
@@ -3528,19 +3528,19 @@
         <v>75010</v>
       </c>
       <c r="E18" t="n">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>58.00626898111504</v>
+        <v>60.86646784106294</v>
       </c>
       <c r="H18" t="n">
-        <v>201.1290322580645</v>
+        <v>206.1157024793388</v>
       </c>
       <c r="I18" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19">
@@ -3561,19 +3561,19 @@
         <v>149990</v>
       </c>
       <c r="E19" t="n">
-        <v>225</v>
+        <v>180</v>
       </c>
       <c r="F19" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="G19" t="n">
-        <v>1134.837767372045</v>
+        <v>1267.427699636192</v>
       </c>
       <c r="H19" t="n">
-        <v>662.5422222222222</v>
+        <v>828.1777777777778</v>
       </c>
       <c r="I19" t="n">
-        <v>420</v>
+        <v>550</v>
       </c>
     </row>
     <row r="20">
@@ -3627,19 +3627,19 @@
         <v>149776</v>
       </c>
       <c r="E21" t="n">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>98.47807930701568</v>
+        <v>96.11030029704173</v>
       </c>
       <c r="H21" t="n">
-        <v>443.2166172106825</v>
+        <v>441.905325443787</v>
       </c>
       <c r="I21" t="n">
-        <v>459</v>
+        <v>458.5</v>
       </c>
     </row>
     <row r="22">
@@ -3693,19 +3693,19 @@
         <v>150000</v>
       </c>
       <c r="E23" t="n">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>96.67824306277116</v>
+        <v>97.4143557481901</v>
       </c>
       <c r="H23" t="n">
-        <v>374.155</v>
+        <v>375.0927318295739</v>
       </c>
       <c r="I23" t="n">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="24">
@@ -4188,19 +4188,19 @@
         <v>149893</v>
       </c>
       <c r="E38" t="n">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="F38" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="G38" t="n">
-        <v>528.7260496662548</v>
+        <v>558.878227453165</v>
       </c>
       <c r="H38" t="n">
-        <v>679.6954545454546</v>
+        <v>708.6872037914692</v>
       </c>
       <c r="I38" t="n">
-        <v>481.5</v>
+        <v>500</v>
       </c>
     </row>
     <row r="39">
@@ -4221,19 +4221,19 @@
         <v>148993</v>
       </c>
       <c r="E39" t="n">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="F39" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G39" t="n">
-        <v>912.5951564368033</v>
+        <v>934.2810369013424</v>
       </c>
       <c r="H39" t="n">
-        <v>477.887459807074</v>
+        <v>497.066889632107</v>
       </c>
       <c r="I39" t="n">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="40">
@@ -4287,19 +4287,19 @@
         <v>150129</v>
       </c>
       <c r="E41" t="n">
-        <v>514</v>
+        <v>504</v>
       </c>
       <c r="F41" t="n">
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>107.1072080868765</v>
+        <v>113.0058232987802</v>
       </c>
       <c r="H41" t="n">
-        <v>291.3599221789883</v>
+        <v>297.140873015873</v>
       </c>
       <c r="I41" t="n">
-        <v>271</v>
+        <v>272.5</v>
       </c>
     </row>
     <row r="42">
@@ -4326,13 +4326,13 @@
         <v>2</v>
       </c>
       <c r="G42" t="n">
-        <v>96.50601092835234</v>
+        <v>96.17550911361717</v>
       </c>
       <c r="H42" t="n">
         <v>371.0173697270471</v>
       </c>
       <c r="I42" t="n">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="43">
@@ -4353,16 +4353,16 @@
         <v>150113</v>
       </c>
       <c r="E43" t="n">
-        <v>367</v>
+        <v>347</v>
       </c>
       <c r="F43" t="n">
         <v>11</v>
       </c>
       <c r="G43" t="n">
-        <v>207.5989266569108</v>
+        <v>230.0996024319968</v>
       </c>
       <c r="H43" t="n">
-        <v>408.3460490463215</v>
+        <v>431.8818443804034</v>
       </c>
       <c r="I43" t="n">
         <v>350</v>
@@ -4980,16 +4980,16 @@
         <v>149651</v>
       </c>
       <c r="E62" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F62" t="n">
         <v>9</v>
       </c>
       <c r="G62" t="n">
-        <v>181.1948954759931</v>
+        <v>182.7426354039304</v>
       </c>
       <c r="H62" t="n">
-        <v>384.0077120822622</v>
+        <v>384.9974226804124</v>
       </c>
       <c r="I62" t="n">
         <v>348</v>
@@ -5145,19 +5145,19 @@
         <v>87577</v>
       </c>
       <c r="E67" t="n">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="F67" t="n">
         <v>11</v>
       </c>
       <c r="G67" t="n">
-        <v>236.4023270221856</v>
+        <v>242.1079380062508</v>
       </c>
       <c r="H67" t="n">
-        <v>440.9242424242424</v>
+        <v>450.0154639175258</v>
       </c>
       <c r="I67" t="n">
-        <v>364</v>
+        <v>368</v>
       </c>
     </row>
     <row r="68">
@@ -5244,16 +5244,16 @@
         <v>85892</v>
       </c>
       <c r="E70" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F70" t="n">
         <v>7</v>
       </c>
       <c r="G70" t="n">
-        <v>195.1890872788387</v>
+        <v>197.1287605977355</v>
       </c>
       <c r="H70" t="n">
-        <v>440.6839378238342</v>
+        <v>442.9791666666667</v>
       </c>
       <c r="I70" t="n">
         <v>400</v>
@@ -5310,16 +5310,16 @@
         <v>110273</v>
       </c>
       <c r="E72" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G72" t="n">
-        <v>167.9486380349468</v>
+        <v>171.4032928110844</v>
       </c>
       <c r="H72" t="n">
-        <v>390.576512455516</v>
+        <v>391.9714285714286</v>
       </c>
       <c r="I72" t="n">
         <v>380</v>
@@ -5409,19 +5409,19 @@
         <v>103611</v>
       </c>
       <c r="E75" t="n">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F75" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G75" t="n">
-        <v>473.0011999058121</v>
+        <v>501.8004460697151</v>
       </c>
       <c r="H75" t="n">
-        <v>631.4320987654321</v>
+        <v>655.7179487179487</v>
       </c>
       <c r="I75" t="n">
-        <v>461</v>
+        <v>468</v>
       </c>
     </row>
     <row r="76">
@@ -5442,16 +5442,16 @@
         <v>150426</v>
       </c>
       <c r="E76" t="n">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F76" t="n">
         <v>1</v>
       </c>
       <c r="G76" t="n">
-        <v>105.553114007537</v>
+        <v>108.0404269074661</v>
       </c>
       <c r="H76" t="n">
-        <v>418.8966480446927</v>
+        <v>420.0700280112045</v>
       </c>
       <c r="I76" t="n">
         <v>418</v>
@@ -5475,19 +5475,19 @@
         <v>104019</v>
       </c>
       <c r="E77" t="n">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>74.95907155897538</v>
+        <v>83.72047725308828</v>
       </c>
       <c r="H77" t="n">
-        <v>325.7106918238994</v>
+        <v>331.9743589743589</v>
       </c>
       <c r="I77" t="n">
-        <v>305</v>
+        <v>307.5</v>
       </c>
     </row>
     <row r="78">
@@ -6097,16 +6097,16 @@
         <v>74910</v>
       </c>
       <c r="E16" t="n">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>70.23510238134244</v>
+        <v>70.97140094441961</v>
       </c>
       <c r="H16" t="n">
-        <v>220.6863905325444</v>
+        <v>221.3412462908012</v>
       </c>
       <c r="I16" t="n">
         <v>213</v>
@@ -6163,19 +6163,19 @@
         <v>36643</v>
       </c>
       <c r="E18" t="n">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>66.28927834758096</v>
+        <v>72.70855683770228</v>
       </c>
       <c r="H18" t="n">
-        <v>223.7852760736196</v>
+        <v>227.98125</v>
       </c>
       <c r="I18" t="n">
-        <v>211</v>
+        <v>212.5</v>
       </c>
     </row>
     <row r="19">
@@ -6262,19 +6262,19 @@
         <v>75011</v>
       </c>
       <c r="E21" t="n">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>53.44561693295265</v>
+        <v>55.6586394854496</v>
       </c>
       <c r="H21" t="n">
-        <v>228.4709480122324</v>
+        <v>230.5864197530864</v>
       </c>
       <c r="I21" t="n">
-        <v>219</v>
+        <v>219.5</v>
       </c>
     </row>
     <row r="22">
@@ -6295,19 +6295,19 @@
         <v>74707</v>
       </c>
       <c r="E22" t="n">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="F22" t="n">
         <v>13</v>
       </c>
       <c r="G22" t="n">
-        <v>133.3574125741211</v>
+        <v>134.1016973385147</v>
       </c>
       <c r="H22" t="n">
-        <v>240.2225806451613</v>
+        <v>241.7824675324675</v>
       </c>
       <c r="I22" t="n">
-        <v>208.5</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23">
@@ -6361,16 +6361,16 @@
         <v>74948</v>
       </c>
       <c r="E24" t="n">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F24" t="n">
         <v>7</v>
       </c>
       <c r="G24" t="n">
-        <v>111.0912143300063</v>
+        <v>111.4878475482435</v>
       </c>
       <c r="H24" t="n">
-        <v>234.8490566037736</v>
+        <v>235.589905362776</v>
       </c>
       <c r="I24" t="n">
         <v>209</v>
@@ -6718,25 +6718,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>74.497</v>
+        <v>73.944</v>
       </c>
       <c r="D35" t="n">
-        <v>74497</v>
+        <v>73944</v>
       </c>
       <c r="E35" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="F35" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G35" t="n">
-        <v>1292.239490429687</v>
+        <v>1563.379224524659</v>
       </c>
       <c r="H35" t="n">
-        <v>1030.472222222222</v>
+        <v>1315.017857142857</v>
       </c>
       <c r="I35" t="n">
-        <v>570.5</v>
+        <v>921</v>
       </c>
     </row>
     <row r="36">
@@ -6922,16 +6922,16 @@
         <v>74935</v>
       </c>
       <c r="E41" t="n">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>47.50909961870469</v>
+        <v>48.18840693231199</v>
       </c>
       <c r="H41" t="n">
-        <v>207.5722222222222</v>
+        <v>208.150417827298</v>
       </c>
       <c r="I41" t="n">
         <v>200</v>
@@ -7318,16 +7318,16 @@
         <v>74937</v>
       </c>
       <c r="E53" t="n">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="F53" t="n">
         <v>7</v>
       </c>
       <c r="G53" t="n">
-        <v>107.8566192677451</v>
+        <v>109.9169220597693</v>
       </c>
       <c r="H53" t="n">
-        <v>202.7880434782609</v>
+        <v>205.0164835164835</v>
       </c>
       <c r="I53" t="n">
         <v>182</v>
@@ -7351,16 +7351,16 @@
         <v>67766</v>
       </c>
       <c r="E54" t="n">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="F54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G54" t="n">
-        <v>97.65880381253844</v>
+        <v>105.0009089050547</v>
       </c>
       <c r="H54" t="n">
-        <v>224.9533333333333</v>
+        <v>229.5442176870748</v>
       </c>
       <c r="I54" t="n">
         <v>207</v>
@@ -7384,16 +7384,16 @@
         <v>75051</v>
       </c>
       <c r="E55" t="n">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>35.66775881927214</v>
+        <v>35.90978109413391</v>
       </c>
       <c r="H55" t="n">
-        <v>222.4107142857143</v>
+        <v>223.0746268656716</v>
       </c>
       <c r="I55" t="n">
         <v>215</v>
@@ -7417,19 +7417,19 @@
         <v>75110</v>
       </c>
       <c r="E56" t="n">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F56" t="n">
         <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>90.59216429019995</v>
+        <v>90.98849294875833</v>
       </c>
       <c r="H56" t="n">
-        <v>220.2441176470588</v>
+        <v>220.8938053097345</v>
       </c>
       <c r="I56" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="57">
@@ -7576,25 +7576,25 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>93.277</v>
+        <v>93.07899999999999</v>
       </c>
       <c r="D61" t="n">
-        <v>93277</v>
+        <v>93079</v>
       </c>
       <c r="E61" t="n">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F61" t="n">
         <v>3</v>
       </c>
       <c r="G61" t="n">
-        <v>65.68057928751597</v>
+        <v>66.25887165193694</v>
       </c>
       <c r="H61" t="n">
-        <v>248.3306666666667</v>
+        <v>249.1313672922252</v>
       </c>
       <c r="I61" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="62">
@@ -7681,19 +7681,19 @@
         <v>74737</v>
       </c>
       <c r="E64" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F64" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G64" t="n">
-        <v>1464.115850948961</v>
+        <v>1480.665160480356</v>
       </c>
       <c r="H64" t="n">
-        <v>1147.2</v>
+        <v>1165.125</v>
       </c>
       <c r="I64" t="n">
-        <v>569</v>
+        <v>545</v>
       </c>
     </row>
     <row r="65">
@@ -7714,19 +7714,19 @@
         <v>60596</v>
       </c>
       <c r="E65" t="n">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="F65" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G65" t="n">
-        <v>355.5493699108007</v>
+        <v>377.5924749188742</v>
       </c>
       <c r="H65" t="n">
-        <v>438.5182481751825</v>
+        <v>473.0472440944882</v>
       </c>
       <c r="I65" t="n">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="66">
@@ -7747,19 +7747,19 @@
         <v>54365</v>
       </c>
       <c r="E66" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F66" t="n">
         <v>3</v>
       </c>
       <c r="G66" t="n">
-        <v>804.28260528959</v>
+        <v>806.5184284224771</v>
       </c>
       <c r="H66" t="n">
-        <v>289.3529411764706</v>
+        <v>290.9086021505377</v>
       </c>
       <c r="I66" t="n">
-        <v>221</v>
+        <v>221.5</v>
       </c>
     </row>
     <row r="67">
@@ -7774,25 +7774,25 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>49.275</v>
+        <v>49.072</v>
       </c>
       <c r="D67" t="n">
-        <v>49275</v>
+        <v>49072</v>
       </c>
       <c r="E67" t="n">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="F67" t="n">
         <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>872.8591110642532</v>
+        <v>884.8312213364255</v>
       </c>
       <c r="H67" t="n">
-        <v>266.0706521739131</v>
+        <v>272.3687150837989</v>
       </c>
       <c r="I67" t="n">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="68">
@@ -7978,19 +7978,19 @@
         <v>74777</v>
       </c>
       <c r="E73" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F73" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G73" t="n">
-        <v>675.076357179755</v>
+        <v>692.4208167422515</v>
       </c>
       <c r="H73" t="n">
-        <v>731.5353535353536</v>
+        <v>762.3368421052631</v>
       </c>
       <c r="I73" t="n">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="74">
@@ -8171,16 +8171,16 @@
         <v>71763</v>
       </c>
       <c r="E3" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" t="n">
-        <v>240.8748421789677</v>
+        <v>244.9161829264773</v>
       </c>
       <c r="H3" t="n">
-        <v>431.0361445783133</v>
+        <v>433.6484848484848</v>
       </c>
       <c r="I3" t="n">
         <v>368</v>
@@ -8468,19 +8468,19 @@
         <v>74988</v>
       </c>
       <c r="E12" t="n">
-        <v>251</v>
+        <v>225</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>52.91597278042619</v>
+        <v>108.2553415229658</v>
       </c>
       <c r="H12" t="n">
-        <v>297.3784860557769</v>
+        <v>331.7422222222222</v>
       </c>
       <c r="I12" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13">
@@ -8534,19 +8534,19 @@
         <v>75456</v>
       </c>
       <c r="E14" t="n">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F14" t="n">
         <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>210.7842003443518</v>
+        <v>212.0434657539298</v>
       </c>
       <c r="H14" t="n">
-        <v>413.6703296703297</v>
+        <v>415.9558011049724</v>
       </c>
       <c r="I14" t="n">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="15">
@@ -8699,19 +8699,19 @@
         <v>37287</v>
       </c>
       <c r="E19" t="n">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>54.42507140822192</v>
+        <v>64.40473968075548</v>
       </c>
       <c r="H19" t="n">
-        <v>204.9779005524862</v>
+        <v>214.4566473988439</v>
       </c>
       <c r="I19" t="n">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="20">
@@ -8732,19 +8732,19 @@
         <v>74938</v>
       </c>
       <c r="E20" t="n">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>78.2306250592551</v>
+        <v>80.59434885345389</v>
       </c>
       <c r="H20" t="n">
-        <v>391.1937172774869</v>
+        <v>393.2526315789474</v>
       </c>
       <c r="I20" t="n">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21">
@@ -8798,19 +8798,19 @@
         <v>74292</v>
       </c>
       <c r="E22" t="n">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="F22" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G22" t="n">
-        <v>329.5023670714072</v>
+        <v>343.8598824594836</v>
       </c>
       <c r="H22" t="n">
-        <v>463.3375</v>
+        <v>484.5359477124183</v>
       </c>
       <c r="I22" t="n">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="23">
@@ -8864,16 +8864,16 @@
         <v>74851</v>
       </c>
       <c r="E24" t="n">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F24" t="n">
         <v>4</v>
       </c>
       <c r="G24" t="n">
-        <v>162.2630146366878</v>
+        <v>164.2242940045646</v>
       </c>
       <c r="H24" t="n">
-        <v>389.586387434555</v>
+        <v>391.6368421052632</v>
       </c>
       <c r="I24" t="n">
         <v>360</v>
@@ -8897,19 +8897,19 @@
         <v>74805</v>
       </c>
       <c r="E25" t="n">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>122.7639736766612</v>
+        <v>131.5842055163205</v>
       </c>
       <c r="H25" t="n">
-        <v>382.1487179487179</v>
+        <v>390.151832460733</v>
       </c>
       <c r="I25" t="n">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="26">
@@ -9293,19 +9293,19 @@
         <v>74926</v>
       </c>
       <c r="E37" t="n">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="F37" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G37" t="n">
-        <v>227.9476272283228</v>
+        <v>245.5336134557088</v>
       </c>
       <c r="H37" t="n">
-        <v>407.3224043715847</v>
+        <v>425.9428571428571</v>
       </c>
       <c r="I37" t="n">
-        <v>318</v>
+        <v>325</v>
       </c>
     </row>
     <row r="38">
@@ -9326,19 +9326,19 @@
         <v>75112</v>
       </c>
       <c r="E38" t="n">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="F38" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G38" t="n">
-        <v>300.588495456747</v>
+        <v>317.4651104535074</v>
       </c>
       <c r="H38" t="n">
-        <v>462.0987654320988</v>
+        <v>482.9677419354838</v>
       </c>
       <c r="I38" t="n">
-        <v>390</v>
+        <v>402</v>
       </c>
     </row>
     <row r="39">
@@ -9392,16 +9392,16 @@
         <v>74956</v>
       </c>
       <c r="E40" t="n">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="F40" t="n">
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>104.141837793851</v>
+        <v>108.3509123776126</v>
       </c>
       <c r="H40" t="n">
-        <v>272.1642335766423</v>
+        <v>277.2230483271375</v>
       </c>
       <c r="I40" t="n">
         <v>256</v>
@@ -9458,19 +9458,19 @@
         <v>72312</v>
       </c>
       <c r="E42" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G42" t="n">
-        <v>3657.18939670901</v>
+        <v>3789.194692995937</v>
       </c>
       <c r="H42" t="n">
-        <v>1842.076923076923</v>
+        <v>1995.583333333333</v>
       </c>
       <c r="I42" t="n">
-        <v>665</v>
+        <v>697</v>
       </c>
     </row>
     <row r="43">
@@ -9491,19 +9491,19 @@
         <v>74492</v>
       </c>
       <c r="E43" t="n">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F43" t="n">
         <v>11</v>
       </c>
       <c r="G43" t="n">
-        <v>332.7651596502091</v>
+        <v>345.6008135116616</v>
       </c>
       <c r="H43" t="n">
-        <v>504.2721088435374</v>
+        <v>514.7777777777778</v>
       </c>
       <c r="I43" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
     </row>
     <row r="44">
@@ -9722,19 +9722,19 @@
         <v>69142</v>
       </c>
       <c r="E50" t="n">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F50" t="n">
         <v>11</v>
       </c>
       <c r="G50" t="n">
-        <v>471.0593645898543</v>
+        <v>484.0356676316695</v>
       </c>
       <c r="H50" t="n">
-        <v>503.1751824817518</v>
+        <v>526.2213740458016</v>
       </c>
       <c r="I50" t="n">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="51">
@@ -9821,19 +9821,19 @@
         <v>74809</v>
       </c>
       <c r="E53" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F53" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G53" t="n">
-        <v>375.0804985021006</v>
+        <v>379.6282965642991</v>
       </c>
       <c r="H53" t="n">
-        <v>535.2877697841726</v>
+        <v>539.1666666666666</v>
       </c>
       <c r="I53" t="n">
-        <v>355</v>
+        <v>354.5</v>
       </c>
     </row>
     <row r="54">
@@ -9986,19 +9986,19 @@
         <v>74875</v>
       </c>
       <c r="E58" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>136.2567383249071</v>
+        <v>136.4719505901947</v>
       </c>
       <c r="H58" t="n">
-        <v>323.4329004329005</v>
+        <v>323.7434782608696</v>
       </c>
       <c r="I58" t="n">
-        <v>311</v>
+        <v>311.5</v>
       </c>
     </row>
     <row r="59">
@@ -10217,16 +10217,16 @@
         <v>22515</v>
       </c>
       <c r="E65" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F65" t="n">
         <v>2</v>
       </c>
       <c r="G65" t="n">
-        <v>236.5987518727754</v>
+        <v>260.7041066145176</v>
       </c>
       <c r="H65" t="n">
-        <v>449.2244897959184</v>
+        <v>458.5833333333333</v>
       </c>
       <c r="I65" t="n">
         <v>394</v>
@@ -10256,7 +10256,7 @@
         <v>3</v>
       </c>
       <c r="G66" t="n">
-        <v>119.671767416973</v>
+        <v>119.6659502594983</v>
       </c>
       <c r="H66" t="n">
         <v>386.3846153846154</v>
@@ -10349,19 +10349,19 @@
         <v>54225</v>
       </c>
       <c r="E69" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F69" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G69" t="n">
-        <v>773.101480867737</v>
+        <v>778.5223844738139</v>
       </c>
       <c r="H69" t="n">
-        <v>635.0705882352942</v>
+        <v>642.6309523809524</v>
       </c>
       <c r="I69" t="n">
-        <v>397</v>
+        <v>396.5</v>
       </c>
     </row>
     <row r="70">
@@ -10481,19 +10481,19 @@
         <v>52248</v>
       </c>
       <c r="E73" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F73" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G73" t="n">
-        <v>620.8152448162034</v>
+        <v>628.0606939724934</v>
       </c>
       <c r="H73" t="n">
-        <v>645.4625</v>
+        <v>653.632911392405</v>
       </c>
       <c r="I73" t="n">
-        <v>437.5</v>
+        <v>417</v>
       </c>
     </row>
     <row r="74">

</xml_diff>

<commit_message>
finish the analysis pipeline  - using Moritz's interpolation, fixing bugs, and organize the folders
</commit_message>
<xml_diff>
--- a/Best ch pipeline/improved_best_channels_stat.xlsx
+++ b/Best ch pipeline/improved_best_channels_stat.xlsx
@@ -662,19 +662,19 @@
         <v>126453</v>
       </c>
       <c r="E7" t="n">
-        <v>587</v>
+        <v>571</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>54.6846528203046</v>
+        <v>64.89298379302498</v>
       </c>
       <c r="H7" t="n">
-        <v>214.9284497444634</v>
+        <v>220.9509632224168</v>
       </c>
       <c r="I7" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8">
@@ -860,16 +860,16 @@
         <v>150039</v>
       </c>
       <c r="E13" t="n">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>28.4071238299095</v>
+        <v>29.28067948513996</v>
       </c>
       <c r="H13" t="n">
-        <v>219.906020558003</v>
+        <v>220.2294117647059</v>
       </c>
       <c r="I13" t="n">
         <v>220</v>
@@ -926,19 +926,19 @@
         <v>98547</v>
       </c>
       <c r="E15" t="n">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>58.9875155194828</v>
+        <v>61.89551450325581</v>
       </c>
       <c r="H15" t="n">
-        <v>210.5824411134904</v>
+        <v>212.4017278617711</v>
       </c>
       <c r="I15" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16">
@@ -959,16 +959,16 @@
         <v>149857</v>
       </c>
       <c r="E16" t="n">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>29.64543133834556</v>
+        <v>30.57212791340253</v>
       </c>
       <c r="H16" t="n">
-        <v>216.3849493487699</v>
+        <v>216.6985507246377</v>
       </c>
       <c r="I16" t="n">
         <v>212</v>
@@ -992,16 +992,16 @@
         <v>150180</v>
       </c>
       <c r="E17" t="n">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>13.52541688734399</v>
+        <v>15.45621107075249</v>
       </c>
       <c r="H17" t="n">
-        <v>230.9460708782743</v>
+        <v>231.3024691358025</v>
       </c>
       <c r="I17" t="n">
         <v>231</v>
@@ -1091,16 +1091,16 @@
         <v>149986</v>
       </c>
       <c r="E20" t="n">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>17.93873064750624</v>
+        <v>20.44425371667523</v>
       </c>
       <c r="H20" t="n">
-        <v>241.2447665056361</v>
+        <v>241.6338709677419</v>
       </c>
       <c r="I20" t="n">
         <v>239</v>
@@ -1157,16 +1157,16 @@
         <v>150121</v>
       </c>
       <c r="E22" t="n">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="F22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G22" t="n">
-        <v>51.83226834444993</v>
+        <v>59.53722876284785</v>
       </c>
       <c r="H22" t="n">
-        <v>231.2638888888889</v>
+        <v>233.4252336448598</v>
       </c>
       <c r="I22" t="n">
         <v>226</v>
@@ -1190,16 +1190,16 @@
         <v>150091</v>
       </c>
       <c r="E23" t="n">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>15.92528616993352</v>
+        <v>15.93446228876659</v>
       </c>
       <c r="H23" t="n">
-        <v>228.9129770992366</v>
+        <v>228.9250764525994</v>
       </c>
       <c r="I23" t="n">
         <v>227</v>
@@ -1256,16 +1256,16 @@
         <v>149903</v>
       </c>
       <c r="E25" t="n">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="F25" t="n">
         <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>38.96217293991534</v>
+        <v>40.28088914190457</v>
       </c>
       <c r="H25" t="n">
-        <v>214.6886657101865</v>
+        <v>215.3064748201439</v>
       </c>
       <c r="I25" t="n">
         <v>208</v>
@@ -1421,16 +1421,16 @@
         <v>149944</v>
       </c>
       <c r="E30" t="n">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>19.64777886291388</v>
+        <v>20.80295382822854</v>
       </c>
       <c r="H30" t="n">
-        <v>249.3533333333333</v>
+        <v>249.7696160267112</v>
       </c>
       <c r="I30" t="n">
         <v>249</v>
@@ -1454,19 +1454,19 @@
         <v>147485</v>
       </c>
       <c r="E31" t="n">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>27.30335297170842</v>
+        <v>30.6433651171726</v>
       </c>
       <c r="H31" t="n">
-        <v>217.8934911242604</v>
+        <v>219.1904761904762</v>
       </c>
       <c r="I31" t="n">
-        <v>211.5</v>
+        <v>213</v>
       </c>
     </row>
     <row r="32">
@@ -1619,19 +1619,19 @@
         <v>150053</v>
       </c>
       <c r="E36" t="n">
-        <v>524</v>
+        <v>501</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" t="n">
-        <v>665.2150524470057</v>
+        <v>681.274328249155</v>
       </c>
       <c r="H36" t="n">
-        <v>285.7290076335878</v>
+        <v>298.8463073852295</v>
       </c>
       <c r="I36" t="n">
-        <v>239.5</v>
+        <v>242</v>
       </c>
     </row>
     <row r="37">
@@ -1652,19 +1652,19 @@
         <v>147583</v>
       </c>
       <c r="E37" t="n">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="F37" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G37" t="n">
-        <v>1215.649782895623</v>
+        <v>1176.972569985177</v>
       </c>
       <c r="H37" t="n">
-        <v>769.1256544502618</v>
+        <v>730.860696517413</v>
       </c>
       <c r="I37" t="n">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="38">
@@ -1685,16 +1685,16 @@
         <v>150146</v>
       </c>
       <c r="E38" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F38" t="n">
         <v>9</v>
       </c>
       <c r="G38" t="n">
-        <v>165.3760084809848</v>
+        <v>165.6720430706115</v>
       </c>
       <c r="H38" t="n">
-        <v>252.2323232323232</v>
+        <v>251.8084033613445</v>
       </c>
       <c r="I38" t="n">
         <v>215</v>
@@ -1784,16 +1784,16 @@
         <v>150167</v>
       </c>
       <c r="E41" t="n">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F41" t="n">
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>33.01010972315376</v>
+        <v>35.10465175569255</v>
       </c>
       <c r="H41" t="n">
-        <v>215.8489208633094</v>
+        <v>216.1599423631124</v>
       </c>
       <c r="I41" t="n">
         <v>213</v>
@@ -1949,16 +1949,16 @@
         <v>149658</v>
       </c>
       <c r="E46" t="n">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="F46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G46" t="n">
-        <v>38.2053742037219</v>
+        <v>42.48000158272951</v>
       </c>
       <c r="H46" t="n">
-        <v>223.3243647234679</v>
+        <v>224.6676691729323</v>
       </c>
       <c r="I46" t="n">
         <v>220</v>
@@ -2048,16 +2048,16 @@
         <v>150096</v>
       </c>
       <c r="E49" t="n">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>18.19312115352909</v>
+        <v>25.63024826616896</v>
       </c>
       <c r="H49" t="n">
-        <v>235.5298742138365</v>
+        <v>236.2728706624606</v>
       </c>
       <c r="I49" t="n">
         <v>235</v>
@@ -2081,19 +2081,19 @@
         <v>150072</v>
       </c>
       <c r="E50" t="n">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>23.56469082649877</v>
+        <v>24.74771818080553</v>
       </c>
       <c r="H50" t="n">
-        <v>236.5797788309637</v>
+        <v>236.9541139240506</v>
       </c>
       <c r="I50" t="n">
-        <v>233</v>
+        <v>233.5</v>
       </c>
     </row>
     <row r="51">
@@ -2114,16 +2114,16 @@
         <v>150098</v>
       </c>
       <c r="E51" t="n">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>31.9241891159244</v>
+        <v>32.8364515129869</v>
       </c>
       <c r="H51" t="n">
-        <v>245.8131147540984</v>
+        <v>246.2167487684729</v>
       </c>
       <c r="I51" t="n">
         <v>243</v>
@@ -2180,16 +2180,16 @@
         <v>150076</v>
       </c>
       <c r="E53" t="n">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>18.1930575677453</v>
+        <v>20.66477369956011</v>
       </c>
       <c r="H53" t="n">
-        <v>218.6788321167883</v>
+        <v>219.3191800878477</v>
       </c>
       <c r="I53" t="n">
         <v>217</v>
@@ -2213,16 +2213,16 @@
         <v>150398</v>
       </c>
       <c r="E54" t="n">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>11.13204116542215</v>
+        <v>12.55901381616846</v>
       </c>
       <c r="H54" t="n">
-        <v>209.677374301676</v>
+        <v>209.9706293706294</v>
       </c>
       <c r="I54" t="n">
         <v>209</v>
@@ -2312,16 +2312,16 @@
         <v>149964</v>
       </c>
       <c r="E57" t="n">
-        <v>709</v>
+        <v>699</v>
       </c>
       <c r="F57" t="n">
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>33.65055211301559</v>
+        <v>42.5931376559976</v>
       </c>
       <c r="H57" t="n">
-        <v>211.1086036671368</v>
+        <v>214.1287553648069</v>
       </c>
       <c r="I57" t="n">
         <v>208</v>
@@ -2345,19 +2345,19 @@
         <v>150089</v>
       </c>
       <c r="E58" t="n">
-        <v>642</v>
+        <v>633</v>
       </c>
       <c r="F58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G58" t="n">
-        <v>73.90515916143966</v>
+        <v>79.46038221448578</v>
       </c>
       <c r="H58" t="n">
-        <v>233.2834890965732</v>
+        <v>236.6003159557662</v>
       </c>
       <c r="I58" t="n">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="59">
@@ -2609,16 +2609,16 @@
         <v>71603</v>
       </c>
       <c r="E66" t="n">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="F66" t="n">
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>43.83932431832092</v>
+        <v>54.58901582722785</v>
       </c>
       <c r="H66" t="n">
-        <v>219.8672839506173</v>
+        <v>225.4335443037975</v>
       </c>
       <c r="I66" t="n">
         <v>216</v>
@@ -2675,19 +2675,19 @@
         <v>85908</v>
       </c>
       <c r="E68" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F68" t="n">
         <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>38.93686729135707</v>
+        <v>39.95664232508493</v>
       </c>
       <c r="H68" t="n">
-        <v>223.0625</v>
+        <v>223.644908616188</v>
       </c>
       <c r="I68" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="69">
@@ -2708,16 +2708,16 @@
         <v>110120</v>
       </c>
       <c r="E69" t="n">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="F69" t="n">
         <v>3</v>
       </c>
       <c r="G69" t="n">
-        <v>84.10424543944512</v>
+        <v>85.7225856311847</v>
       </c>
       <c r="H69" t="n">
-        <v>251.2929061784897</v>
+        <v>253.0299539170507</v>
       </c>
       <c r="I69" t="n">
         <v>240</v>
@@ -2807,16 +2807,16 @@
         <v>150466</v>
       </c>
       <c r="E72" t="n">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="F72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G72" t="n">
-        <v>32.11988502964557</v>
+        <v>36.23309475170235</v>
       </c>
       <c r="H72" t="n">
-        <v>223.5044642857143</v>
+        <v>224.5067264573991</v>
       </c>
       <c r="I72" t="n">
         <v>221</v>
@@ -3330,16 +3330,16 @@
         <v>149707</v>
       </c>
       <c r="E12" t="n">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>103.8239033513958</v>
+        <v>111.405862676011</v>
       </c>
       <c r="H12" t="n">
-        <v>331.1019955654102</v>
+        <v>336.322072072072</v>
       </c>
       <c r="I12" t="n">
         <v>304</v>
@@ -3363,16 +3363,16 @@
         <v>150176</v>
       </c>
       <c r="E13" t="n">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>30.09764129601798</v>
+        <v>33.31200012768191</v>
       </c>
       <c r="H13" t="n">
-        <v>296.0849802371541</v>
+        <v>296.6712871287129</v>
       </c>
       <c r="I13" t="n">
         <v>290</v>
@@ -3396,19 +3396,19 @@
         <v>149498</v>
       </c>
       <c r="E14" t="n">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G14" t="n">
-        <v>160.6564431564435</v>
+        <v>166.4368002877623</v>
       </c>
       <c r="H14" t="n">
-        <v>454.3780487804878</v>
+        <v>458.5723076923077</v>
       </c>
       <c r="I14" t="n">
-        <v>484.5</v>
+        <v>487</v>
       </c>
     </row>
     <row r="15">
@@ -3429,16 +3429,16 @@
         <v>98601</v>
       </c>
       <c r="E15" t="n">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G15" t="n">
-        <v>239.8865782982235</v>
+        <v>245.029812754053</v>
       </c>
       <c r="H15" t="n">
-        <v>436.1741071428572</v>
+        <v>438.1300448430493</v>
       </c>
       <c r="I15" t="n">
         <v>371</v>
@@ -3495,19 +3495,19 @@
         <v>149995</v>
       </c>
       <c r="E17" t="n">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>109.0860371641015</v>
+        <v>126.1080253720491</v>
       </c>
       <c r="H17" t="n">
-        <v>450.0993975903614</v>
+        <v>458.3834355828221</v>
       </c>
       <c r="I17" t="n">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="18">
@@ -3528,19 +3528,19 @@
         <v>75010</v>
       </c>
       <c r="E18" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>60.86646784106294</v>
+        <v>62.06016439157262</v>
       </c>
       <c r="H18" t="n">
-        <v>206.1157024793388</v>
+        <v>207.2576177285319</v>
       </c>
       <c r="I18" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="19">
@@ -3561,19 +3561,19 @@
         <v>149990</v>
       </c>
       <c r="E19" t="n">
-        <v>180</v>
+        <v>202</v>
       </c>
       <c r="F19" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="G19" t="n">
-        <v>1267.427699636192</v>
+        <v>1191.731387980726</v>
       </c>
       <c r="H19" t="n">
-        <v>828.1777777777778</v>
+        <v>737.9801980198019</v>
       </c>
       <c r="I19" t="n">
-        <v>550</v>
+        <v>441.5</v>
       </c>
     </row>
     <row r="20">
@@ -3627,19 +3627,19 @@
         <v>149776</v>
       </c>
       <c r="E21" t="n">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>96.11030029704173</v>
+        <v>103.3312457973396</v>
       </c>
       <c r="H21" t="n">
-        <v>441.905325443787</v>
+        <v>445.8626865671642</v>
       </c>
       <c r="I21" t="n">
-        <v>458.5</v>
+        <v>460</v>
       </c>
     </row>
     <row r="22">
@@ -3660,19 +3660,19 @@
         <v>150094</v>
       </c>
       <c r="E22" t="n">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>81.44196434254106</v>
+        <v>94.14519453145998</v>
       </c>
       <c r="H22" t="n">
-        <v>391.3185378590078</v>
+        <v>397.5464190981432</v>
       </c>
       <c r="I22" t="n">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="23">
@@ -3693,19 +3693,19 @@
         <v>150000</v>
       </c>
       <c r="E23" t="n">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>97.4143557481901</v>
+        <v>104.4355172190794</v>
       </c>
       <c r="H23" t="n">
-        <v>375.0927318295739</v>
+        <v>379.8527918781726</v>
       </c>
       <c r="I23" t="n">
-        <v>372</v>
+        <v>373.5</v>
       </c>
     </row>
     <row r="24">
@@ -3852,22 +3852,22 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>150.181</v>
+        <v>149.701</v>
       </c>
       <c r="D28" t="n">
-        <v>150181</v>
+        <v>149701</v>
       </c>
       <c r="E28" t="n">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>62.47033126328356</v>
+        <v>62.57124312015734</v>
       </c>
       <c r="H28" t="n">
-        <v>481.8745980707395</v>
+        <v>481.8806451612903</v>
       </c>
       <c r="I28" t="n">
         <v>498</v>
@@ -3957,19 +3957,19 @@
         <v>147216</v>
       </c>
       <c r="E31" t="n">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>124.7405834291838</v>
+        <v>129.0272243318418</v>
       </c>
       <c r="H31" t="n">
-        <v>418.3789173789174</v>
+        <v>420.7765042979943</v>
       </c>
       <c r="I31" t="n">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="32">
@@ -3990,16 +3990,16 @@
         <v>145785</v>
       </c>
       <c r="E32" t="n">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>48.32103884563151</v>
+        <v>51.57055749699509</v>
       </c>
       <c r="H32" t="n">
-        <v>332.9610983981693</v>
+        <v>334.4919540229885</v>
       </c>
       <c r="I32" t="n">
         <v>328</v>
@@ -4023,16 +4023,16 @@
         <v>149777</v>
       </c>
       <c r="E33" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>91.34030066883317</v>
+        <v>95.40185836257587</v>
       </c>
       <c r="H33" t="n">
-        <v>388.8046875</v>
+        <v>389.8198433420366</v>
       </c>
       <c r="I33" t="n">
         <v>374</v>
@@ -4188,19 +4188,19 @@
         <v>149893</v>
       </c>
       <c r="E38" t="n">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F38" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G38" t="n">
-        <v>558.878227453165</v>
+        <v>545.0928144788147</v>
       </c>
       <c r="H38" t="n">
-        <v>708.6872037914692</v>
+        <v>695.5023255813953</v>
       </c>
       <c r="I38" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="39">
@@ -4221,19 +4221,19 @@
         <v>148993</v>
       </c>
       <c r="E39" t="n">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="F39" t="n">
         <v>17</v>
       </c>
       <c r="G39" t="n">
-        <v>934.2810369013424</v>
+        <v>923.6923348342572</v>
       </c>
       <c r="H39" t="n">
-        <v>497.066889632107</v>
+        <v>488.891447368421</v>
       </c>
       <c r="I39" t="n">
-        <v>338</v>
+        <v>339.5</v>
       </c>
     </row>
     <row r="40">
@@ -4287,19 +4287,19 @@
         <v>150129</v>
       </c>
       <c r="E41" t="n">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="F41" t="n">
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>113.0058232987802</v>
+        <v>119.2392959805209</v>
       </c>
       <c r="H41" t="n">
-        <v>297.140873015873</v>
+        <v>301.9334677419355</v>
       </c>
       <c r="I41" t="n">
-        <v>272.5</v>
+        <v>273</v>
       </c>
     </row>
     <row r="42">
@@ -4320,19 +4320,19 @@
         <v>149876</v>
       </c>
       <c r="E42" t="n">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="F42" t="n">
         <v>2</v>
       </c>
       <c r="G42" t="n">
-        <v>96.17550911361717</v>
+        <v>102.8406071364346</v>
       </c>
       <c r="H42" t="n">
-        <v>371.0173697270471</v>
+        <v>373.8</v>
       </c>
       <c r="I42" t="n">
-        <v>358</v>
+        <v>358.5</v>
       </c>
     </row>
     <row r="43">
@@ -4353,19 +4353,19 @@
         <v>150113</v>
       </c>
       <c r="E43" t="n">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="F43" t="n">
         <v>11</v>
       </c>
       <c r="G43" t="n">
-        <v>230.0996024319968</v>
+        <v>227.9394062494857</v>
       </c>
       <c r="H43" t="n">
-        <v>431.8818443804034</v>
+        <v>423.3418079096045</v>
       </c>
       <c r="I43" t="n">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="44">
@@ -4380,22 +4380,22 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>150.183</v>
+        <v>149.876</v>
       </c>
       <c r="D44" t="n">
-        <v>150183</v>
+        <v>149876</v>
       </c>
       <c r="E44" t="n">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>21.77551067090279</v>
+        <v>21.74960990530465</v>
       </c>
       <c r="H44" t="n">
-        <v>338.1309255079007</v>
+        <v>338.2013574660634</v>
       </c>
       <c r="I44" t="n">
         <v>337</v>
@@ -4419,16 +4419,16 @@
         <v>150299</v>
       </c>
       <c r="E45" t="n">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F45" t="n">
         <v>4</v>
       </c>
       <c r="G45" t="n">
-        <v>256.6297865646743</v>
+        <v>272.34108356561</v>
       </c>
       <c r="H45" t="n">
-        <v>405.0297297297298</v>
+        <v>406.1273712737128</v>
       </c>
       <c r="I45" t="n">
         <v>388</v>
@@ -4491,7 +4491,7 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>28.99407850399134</v>
+        <v>28.51007909452076</v>
       </c>
       <c r="H47" t="n">
         <v>402.4756756756757</v>
@@ -4617,16 +4617,16 @@
         <v>150037</v>
       </c>
       <c r="E51" t="n">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>58.47606432574423</v>
+        <v>61.54596651784109</v>
       </c>
       <c r="H51" t="n">
-        <v>324.6334056399132</v>
+        <v>326.0479302832244</v>
       </c>
       <c r="I51" t="n">
         <v>316</v>
@@ -4650,16 +4650,16 @@
         <v>150124</v>
       </c>
       <c r="E52" t="n">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>38.87975179378721</v>
+        <v>42.60709344362315</v>
       </c>
       <c r="H52" t="n">
-        <v>337.5382882882883</v>
+        <v>338.3002257336343</v>
       </c>
       <c r="I52" t="n">
         <v>338</v>
@@ -4716,16 +4716,16 @@
         <v>149888</v>
       </c>
       <c r="E54" t="n">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F54" t="n">
         <v>2</v>
       </c>
       <c r="G54" t="n">
-        <v>75.04568535324225</v>
+        <v>77.39574936616432</v>
       </c>
       <c r="H54" t="n">
-        <v>372.1741293532338</v>
+        <v>373.1022443890274</v>
       </c>
       <c r="I54" t="n">
         <v>368</v>
@@ -4749,19 +4749,19 @@
         <v>150014</v>
       </c>
       <c r="E55" t="n">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>61.70622062561102</v>
+        <v>65.35297341608674</v>
       </c>
       <c r="H55" t="n">
-        <v>414.4016620498615</v>
+        <v>415.5527777777778</v>
       </c>
       <c r="I55" t="n">
-        <v>419</v>
+        <v>419.5</v>
       </c>
     </row>
     <row r="56">
@@ -4782,19 +4782,19 @@
         <v>149772</v>
       </c>
       <c r="E56" t="n">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>24.96976863372452</v>
+        <v>27.55869064246772</v>
       </c>
       <c r="H56" t="n">
-        <v>341.9221967963387</v>
+        <v>342.7064220183486</v>
       </c>
       <c r="I56" t="n">
-        <v>344</v>
+        <v>344.5</v>
       </c>
     </row>
     <row r="57">
@@ -4815,19 +4815,19 @@
         <v>150199</v>
       </c>
       <c r="E57" t="n">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="F57" t="n">
         <v>4</v>
       </c>
       <c r="G57" t="n">
-        <v>132.8059191911409</v>
+        <v>134.880321145915</v>
       </c>
       <c r="H57" t="n">
-        <v>366.359413202934</v>
+        <v>368.1597051597051</v>
       </c>
       <c r="I57" t="n">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="58">
@@ -4848,16 +4848,16 @@
         <v>149747</v>
       </c>
       <c r="E58" t="n">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F58" t="n">
         <v>5</v>
       </c>
       <c r="G58" t="n">
-        <v>214.037860859723</v>
+        <v>215.517727699596</v>
       </c>
       <c r="H58" t="n">
-        <v>423.1643059490085</v>
+        <v>424.3664772727273</v>
       </c>
       <c r="I58" t="n">
         <v>407</v>
@@ -4881,19 +4881,19 @@
         <v>149976</v>
       </c>
       <c r="E59" t="n">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="F59" t="n">
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>45.64489881512876</v>
+        <v>56.14639142541599</v>
       </c>
       <c r="H59" t="n">
-        <v>338.6651583710407</v>
+        <v>341.7579908675799</v>
       </c>
       <c r="I59" t="n">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="60">
@@ -4914,19 +4914,19 @@
         <v>150182</v>
       </c>
       <c r="E60" t="n">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>24.33740636095625</v>
+        <v>42.80872884818174</v>
       </c>
       <c r="H60" t="n">
-        <v>396.6772486772487</v>
+        <v>399.8506666666667</v>
       </c>
       <c r="I60" t="n">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="61">
@@ -5079,19 +5079,19 @@
         <v>150185</v>
       </c>
       <c r="E65" t="n">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="F65" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G65" t="n">
-        <v>160.9776735948541</v>
+        <v>174.0201388120507</v>
       </c>
       <c r="H65" t="n">
-        <v>427.3019943019943</v>
+        <v>432.2276657060519</v>
       </c>
       <c r="I65" t="n">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="66">
@@ -5112,16 +5112,16 @@
         <v>150171</v>
       </c>
       <c r="E66" t="n">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F66" t="n">
         <v>2</v>
       </c>
       <c r="G66" t="n">
-        <v>111.5952605640657</v>
+        <v>113.0113110426356</v>
       </c>
       <c r="H66" t="n">
-        <v>390.9791122715405</v>
+        <v>392.0026178010471</v>
       </c>
       <c r="I66" t="n">
         <v>378</v>
@@ -5211,19 +5211,19 @@
         <v>60132</v>
       </c>
       <c r="E69" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>65.79395256421776</v>
+        <v>72.43165227611115</v>
       </c>
       <c r="H69" t="n">
-        <v>380.1656050955414</v>
+        <v>382.6025641025641</v>
       </c>
       <c r="I69" t="n">
-        <v>376</v>
+        <v>376.5</v>
       </c>
     </row>
     <row r="70">
@@ -5244,16 +5244,16 @@
         <v>85892</v>
       </c>
       <c r="E70" t="n">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F70" t="n">
         <v>7</v>
       </c>
       <c r="G70" t="n">
-        <v>197.1287605977355</v>
+        <v>199.1756959059645</v>
       </c>
       <c r="H70" t="n">
-        <v>442.9791666666667</v>
+        <v>445.2984293193717</v>
       </c>
       <c r="I70" t="n">
         <v>400</v>
@@ -5310,19 +5310,19 @@
         <v>110273</v>
       </c>
       <c r="E72" t="n">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="F72" t="n">
         <v>3</v>
       </c>
       <c r="G72" t="n">
-        <v>171.4032928110844</v>
+        <v>180.5356061433419</v>
       </c>
       <c r="H72" t="n">
-        <v>391.9714285714286</v>
+        <v>396.2166064981949</v>
       </c>
       <c r="I72" t="n">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="73">
@@ -5376,16 +5376,16 @@
         <v>149955</v>
       </c>
       <c r="E74" t="n">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="F74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G74" t="n">
-        <v>92.42117509108674</v>
+        <v>100.8022544663288</v>
       </c>
       <c r="H74" t="n">
-        <v>407.9645776566758</v>
+        <v>410.2</v>
       </c>
       <c r="I74" t="n">
         <v>393</v>
@@ -5409,19 +5409,19 @@
         <v>103611</v>
       </c>
       <c r="E75" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F75" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G75" t="n">
-        <v>501.8004460697151</v>
+        <v>487.9783488878481</v>
       </c>
       <c r="H75" t="n">
-        <v>655.7179487179487</v>
+        <v>647.4177215189874</v>
       </c>
       <c r="I75" t="n">
-        <v>468</v>
+        <v>469.5</v>
       </c>
     </row>
     <row r="76">
@@ -5442,19 +5442,19 @@
         <v>150426</v>
       </c>
       <c r="E76" t="n">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="F76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>108.0404269074661</v>
+        <v>123.1061555536746</v>
       </c>
       <c r="H76" t="n">
-        <v>420.0700280112045</v>
+        <v>427.2507122507122</v>
       </c>
       <c r="I76" t="n">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="77">
@@ -5475,19 +5475,19 @@
         <v>104019</v>
       </c>
       <c r="E77" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>83.72047725308828</v>
+        <v>83.68154798326962</v>
       </c>
       <c r="H77" t="n">
-        <v>331.9743589743589</v>
+        <v>333.0418006430868</v>
       </c>
       <c r="I77" t="n">
-        <v>307.5</v>
+        <v>308</v>
       </c>
     </row>
     <row r="78">
@@ -5767,19 +5767,19 @@
         <v>75120</v>
       </c>
       <c r="E6" t="n">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>21.11514336623256</v>
+        <v>26.86362974964797</v>
       </c>
       <c r="H6" t="n">
-        <v>209.0474860335196</v>
+        <v>210.8140845070423</v>
       </c>
       <c r="I6" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7">
@@ -5800,19 +5800,19 @@
         <v>74953</v>
       </c>
       <c r="E7" t="n">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>33.46245463632285</v>
+        <v>44.22587111837565</v>
       </c>
       <c r="H7" t="n">
-        <v>217.7026239067055</v>
+        <v>223.5688622754491</v>
       </c>
       <c r="I7" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8">
@@ -6064,19 +6064,19 @@
         <v>74991</v>
       </c>
       <c r="E15" t="n">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>38.57025523773909</v>
+        <v>40.3259121874269</v>
       </c>
       <c r="H15" t="n">
-        <v>207.3102493074792</v>
+        <v>207.8861111111111</v>
       </c>
       <c r="I15" t="n">
-        <v>199</v>
+        <v>199.5</v>
       </c>
     </row>
     <row r="16">
@@ -6130,16 +6130,16 @@
         <v>74997</v>
       </c>
       <c r="E17" t="n">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>8.896344184231122</v>
+        <v>14.59417894975096</v>
       </c>
       <c r="H17" t="n">
-        <v>236.9111111111111</v>
+        <v>237.6656050955414</v>
       </c>
       <c r="I17" t="n">
         <v>237</v>
@@ -6163,19 +6163,19 @@
         <v>36643</v>
       </c>
       <c r="E18" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>72.70855683770228</v>
+        <v>74.11582638064546</v>
       </c>
       <c r="H18" t="n">
-        <v>227.98125</v>
+        <v>229.4150943396226</v>
       </c>
       <c r="I18" t="n">
-        <v>212.5</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19">
@@ -6262,19 +6262,19 @@
         <v>75011</v>
       </c>
       <c r="E21" t="n">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>55.6586394854496</v>
+        <v>61.70412108757429</v>
       </c>
       <c r="H21" t="n">
-        <v>230.5864197530864</v>
+        <v>232.7414330218068</v>
       </c>
       <c r="I21" t="n">
-        <v>219.5</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22">
@@ -6295,16 +6295,16 @@
         <v>74707</v>
       </c>
       <c r="E22" t="n">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F22" t="n">
         <v>13</v>
       </c>
       <c r="G22" t="n">
-        <v>134.1016973385147</v>
+        <v>138.750546796799</v>
       </c>
       <c r="H22" t="n">
-        <v>241.7824675324675</v>
+        <v>244.1606557377049</v>
       </c>
       <c r="I22" t="n">
         <v>209</v>
@@ -6361,16 +6361,16 @@
         <v>74948</v>
       </c>
       <c r="E24" t="n">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G24" t="n">
-        <v>111.4878475482435</v>
+        <v>114.7789379413361</v>
       </c>
       <c r="H24" t="n">
-        <v>235.589905362776</v>
+        <v>237.8407643312102</v>
       </c>
       <c r="I24" t="n">
         <v>209</v>
@@ -6427,16 +6427,16 @@
         <v>74939</v>
       </c>
       <c r="E26" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F26" t="n">
         <v>7</v>
       </c>
       <c r="G26" t="n">
-        <v>85.68908811985834</v>
+        <v>86.70031265253212</v>
       </c>
       <c r="H26" t="n">
-        <v>248.0132890365448</v>
+        <v>248.84</v>
       </c>
       <c r="I26" t="n">
         <v>233</v>
@@ -6499,13 +6499,13 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>21.61996367987969</v>
+        <v>20.12764130651092</v>
       </c>
       <c r="H28" t="n">
         <v>223.9559471365639</v>
       </c>
       <c r="I28" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="29">
@@ -6559,16 +6559,16 @@
         <v>74916</v>
       </c>
       <c r="E30" t="n">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>20.93502582155169</v>
+        <v>32.15363899395697</v>
       </c>
       <c r="H30" t="n">
-        <v>245.733552631579</v>
+        <v>248.1827242524917</v>
       </c>
       <c r="I30" t="n">
         <v>243</v>
@@ -6658,16 +6658,16 @@
         <v>75100</v>
       </c>
       <c r="E33" t="n">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>22.47857054034705</v>
+        <v>33.29176127009173</v>
       </c>
       <c r="H33" t="n">
-        <v>178.8424821002387</v>
+        <v>182.323600973236</v>
       </c>
       <c r="I33" t="n">
         <v>175</v>
@@ -6691,16 +6691,16 @@
         <v>71380</v>
       </c>
       <c r="E34" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>36.29587612941784</v>
+        <v>37.63342733094223</v>
       </c>
       <c r="H34" t="n">
-        <v>231.9609120521173</v>
+        <v>232.718954248366</v>
       </c>
       <c r="I34" t="n">
         <v>232</v>
@@ -6718,25 +6718,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>73.944</v>
+        <v>74.497</v>
       </c>
       <c r="D35" t="n">
-        <v>73944</v>
+        <v>74497</v>
       </c>
       <c r="E35" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="F35" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="G35" t="n">
-        <v>1563.379224524659</v>
+        <v>1314.241302445467</v>
       </c>
       <c r="H35" t="n">
-        <v>1315.017857142857</v>
+        <v>1091.088235294118</v>
       </c>
       <c r="I35" t="n">
-        <v>921</v>
+        <v>750.5</v>
       </c>
     </row>
     <row r="36">
@@ -6757,19 +6757,19 @@
         <v>15992</v>
       </c>
       <c r="E36" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>128.2402281176248</v>
+        <v>132.9267293073696</v>
       </c>
       <c r="H36" t="n">
-        <v>224.7428571428571</v>
+        <v>231.3529411764706</v>
       </c>
       <c r="I36" t="n">
-        <v>204.5</v>
+        <v>205</v>
       </c>
     </row>
     <row r="37">
@@ -6889,19 +6889,19 @@
         <v>64420</v>
       </c>
       <c r="E40" t="n">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>29.52529002278162</v>
+        <v>34.97694119669264</v>
       </c>
       <c r="H40" t="n">
-        <v>237.4</v>
+        <v>240.0674157303371</v>
       </c>
       <c r="I40" t="n">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41">
@@ -6922,16 +6922,16 @@
         <v>74935</v>
       </c>
       <c r="E41" t="n">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>48.18840693231199</v>
+        <v>53.43261526548956</v>
       </c>
       <c r="H41" t="n">
-        <v>208.150417827298</v>
+        <v>209.9044943820225</v>
       </c>
       <c r="I41" t="n">
         <v>200</v>
@@ -6955,19 +6955,19 @@
         <v>74964</v>
       </c>
       <c r="E42" t="n">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>23.23223358000662</v>
+        <v>25.53643554662714</v>
       </c>
       <c r="H42" t="n">
-        <v>233.5</v>
+        <v>234.2319749216301</v>
       </c>
       <c r="I42" t="n">
-        <v>231.5</v>
+        <v>232</v>
       </c>
     </row>
     <row r="43">
@@ -7186,19 +7186,19 @@
         <v>69418</v>
       </c>
       <c r="E49" t="n">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>21.94262899301834</v>
+        <v>26.50216451058444</v>
       </c>
       <c r="H49" t="n">
-        <v>214.8850931677019</v>
+        <v>216.228125</v>
       </c>
       <c r="I49" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="50">
@@ -7252,19 +7252,19 @@
         <v>75057</v>
       </c>
       <c r="E51" t="n">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>23.62265614647264</v>
+        <v>28.56056070362813</v>
       </c>
       <c r="H51" t="n">
-        <v>203.7493188010899</v>
+        <v>205.4285714285714</v>
       </c>
       <c r="I51" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="52">
@@ -7285,19 +7285,19 @@
         <v>68743</v>
       </c>
       <c r="E52" t="n">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>32.00838002774287</v>
+        <v>35.24417134424985</v>
       </c>
       <c r="H52" t="n">
-        <v>199.6355685131195</v>
+        <v>201.3970588235294</v>
       </c>
       <c r="I52" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="53">
@@ -7318,19 +7318,19 @@
         <v>74937</v>
       </c>
       <c r="E53" t="n">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="F53" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G53" t="n">
-        <v>109.9169220597693</v>
+        <v>113.120868491494</v>
       </c>
       <c r="H53" t="n">
-        <v>205.0164835164835</v>
+        <v>207.2944444444445</v>
       </c>
       <c r="I53" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="54">
@@ -7351,16 +7351,16 @@
         <v>67766</v>
       </c>
       <c r="E54" t="n">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="F54" t="n">
         <v>3</v>
       </c>
       <c r="G54" t="n">
-        <v>105.0009089050547</v>
+        <v>107.5600054871617</v>
       </c>
       <c r="H54" t="n">
-        <v>229.5442176870748</v>
+        <v>231.1164383561644</v>
       </c>
       <c r="I54" t="n">
         <v>207</v>
@@ -7384,19 +7384,19 @@
         <v>75051</v>
       </c>
       <c r="E55" t="n">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>35.90978109413391</v>
+        <v>47.93921704997082</v>
       </c>
       <c r="H55" t="n">
-        <v>223.0746268656716</v>
+        <v>227.8353658536585</v>
       </c>
       <c r="I55" t="n">
-        <v>215</v>
+        <v>215.5</v>
       </c>
     </row>
     <row r="56">
@@ -7417,16 +7417,16 @@
         <v>75110</v>
       </c>
       <c r="E56" t="n">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F56" t="n">
         <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>90.98849294875833</v>
+        <v>92.13684944152692</v>
       </c>
       <c r="H56" t="n">
-        <v>220.8938053097345</v>
+        <v>222.2047477744807</v>
       </c>
       <c r="I56" t="n">
         <v>202</v>
@@ -7549,16 +7549,16 @@
         <v>74996</v>
       </c>
       <c r="E60" t="n">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>14.40878044580052</v>
+        <v>17.65929530677977</v>
       </c>
       <c r="H60" t="n">
-        <v>222.0118694362018</v>
+        <v>222.672619047619</v>
       </c>
       <c r="I60" t="n">
         <v>220</v>
@@ -7582,16 +7582,16 @@
         <v>93079</v>
       </c>
       <c r="E61" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F61" t="n">
         <v>3</v>
       </c>
       <c r="G61" t="n">
-        <v>66.25887165193694</v>
+        <v>67.29144239697155</v>
       </c>
       <c r="H61" t="n">
-        <v>249.1313672922252</v>
+        <v>249.8010752688172</v>
       </c>
       <c r="I61" t="n">
         <v>242</v>
@@ -7681,19 +7681,19 @@
         <v>74737</v>
       </c>
       <c r="E64" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F64" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G64" t="n">
-        <v>1480.665160480356</v>
+        <v>1464.115850948961</v>
       </c>
       <c r="H64" t="n">
-        <v>1165.125</v>
+        <v>1147.2</v>
       </c>
       <c r="I64" t="n">
-        <v>545</v>
+        <v>569</v>
       </c>
     </row>
     <row r="65">
@@ -7714,19 +7714,19 @@
         <v>60596</v>
       </c>
       <c r="E65" t="n">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="F65" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="G65" t="n">
-        <v>377.5924749188742</v>
+        <v>363.88972420044</v>
       </c>
       <c r="H65" t="n">
-        <v>473.0472440944882</v>
+        <v>455.1287878787879</v>
       </c>
       <c r="I65" t="n">
-        <v>314</v>
+        <v>316.5</v>
       </c>
     </row>
     <row r="66">
@@ -7774,22 +7774,22 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>49.072</v>
+        <v>49.275</v>
       </c>
       <c r="D67" t="n">
-        <v>49072</v>
+        <v>49275</v>
       </c>
       <c r="E67" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F67" t="n">
         <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>884.8312213364255</v>
+        <v>882.3713128830078</v>
       </c>
       <c r="H67" t="n">
-        <v>272.3687150837989</v>
+        <v>271.9833333333333</v>
       </c>
       <c r="I67" t="n">
         <v>192</v>
@@ -7813,16 +7813,16 @@
         <v>41504</v>
       </c>
       <c r="E68" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G68" t="n">
-        <v>63.17475212483871</v>
+        <v>71.78638839645166</v>
       </c>
       <c r="H68" t="n">
-        <v>254.7160493827161</v>
+        <v>256.2981366459628</v>
       </c>
       <c r="I68" t="n">
         <v>250</v>
@@ -7846,16 +7846,16 @@
         <v>75349</v>
       </c>
       <c r="E69" t="n">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>7.974524340164266</v>
+        <v>7.669846280179111</v>
       </c>
       <c r="H69" t="n">
-        <v>217.2109826589596</v>
+        <v>217.3304347826087</v>
       </c>
       <c r="I69" t="n">
         <v>217</v>
@@ -7978,19 +7978,19 @@
         <v>74777</v>
       </c>
       <c r="E73" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F73" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G73" t="n">
-        <v>692.4208167422515</v>
+        <v>681.384244315982</v>
       </c>
       <c r="H73" t="n">
-        <v>762.3368421052631</v>
+        <v>746.6185567010309</v>
       </c>
       <c r="I73" t="n">
-        <v>547</v>
+        <v>554</v>
       </c>
     </row>
     <row r="74">
@@ -8336,19 +8336,19 @@
         <v>33841</v>
       </c>
       <c r="E8" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>72.39315022896172</v>
+        <v>74.7478686320264</v>
       </c>
       <c r="H8" t="n">
-        <v>202.777108433735</v>
+        <v>205.25</v>
       </c>
       <c r="I8" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9">
@@ -8369,19 +8369,19 @@
         <v>74738</v>
       </c>
       <c r="E9" t="n">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>104.8176386533141</v>
+        <v>111.0614074552651</v>
       </c>
       <c r="H9" t="n">
-        <v>399.8118279569892</v>
+        <v>404.1576086956522</v>
       </c>
       <c r="I9" t="n">
-        <v>401</v>
+        <v>402.5</v>
       </c>
     </row>
     <row r="10">
@@ -8402,19 +8402,19 @@
         <v>74840</v>
       </c>
       <c r="E10" t="n">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>29.21933090484081</v>
+        <v>45.38646971370223</v>
       </c>
       <c r="H10" t="n">
-        <v>333.0803571428572</v>
+        <v>337.6018099547511</v>
       </c>
       <c r="I10" t="n">
-        <v>329.5</v>
+        <v>331</v>
       </c>
     </row>
     <row r="11">
@@ -8468,16 +8468,16 @@
         <v>74988</v>
       </c>
       <c r="E12" t="n">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>108.2553415229658</v>
+        <v>93.58199939378773</v>
       </c>
       <c r="H12" t="n">
-        <v>331.7422222222222</v>
+        <v>321.7327586206897</v>
       </c>
       <c r="I12" t="n">
         <v>286</v>
@@ -8534,19 +8534,19 @@
         <v>75456</v>
       </c>
       <c r="E14" t="n">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F14" t="n">
         <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>212.0434657539298</v>
+        <v>215.931620668371</v>
       </c>
       <c r="H14" t="n">
-        <v>415.9558011049724</v>
+        <v>418.2666666666667</v>
       </c>
       <c r="I14" t="n">
-        <v>371</v>
+        <v>371.5</v>
       </c>
     </row>
     <row r="15">
@@ -8633,19 +8633,19 @@
         <v>75004</v>
       </c>
       <c r="E17" t="n">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>94.07286426399538</v>
+        <v>110.390709466478</v>
       </c>
       <c r="H17" t="n">
-        <v>430.6127167630058</v>
+        <v>438.2117647058823</v>
       </c>
       <c r="I17" t="n">
-        <v>432</v>
+        <v>436</v>
       </c>
     </row>
     <row r="18">
@@ -8732,16 +8732,16 @@
         <v>74938</v>
       </c>
       <c r="E20" t="n">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>80.59434885345389</v>
+        <v>87.98591521712862</v>
       </c>
       <c r="H20" t="n">
-        <v>393.2526315789474</v>
+        <v>395.3333333333333</v>
       </c>
       <c r="I20" t="n">
         <v>393</v>
@@ -8765,16 +8765,16 @@
         <v>74904</v>
       </c>
       <c r="E21" t="n">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>58.26072956151891</v>
+        <v>64.74022432366402</v>
       </c>
       <c r="H21" t="n">
-        <v>382.3230769230769</v>
+        <v>384.2938144329897</v>
       </c>
       <c r="I21" t="n">
         <v>381</v>
@@ -8798,16 +8798,16 @@
         <v>74292</v>
       </c>
       <c r="E22" t="n">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F22" t="n">
         <v>12</v>
       </c>
       <c r="G22" t="n">
-        <v>343.8598824594836</v>
+        <v>337.0735888184482</v>
       </c>
       <c r="H22" t="n">
-        <v>484.5359477124183</v>
+        <v>472.1910828025478</v>
       </c>
       <c r="I22" t="n">
         <v>347</v>
@@ -8864,16 +8864,16 @@
         <v>74851</v>
       </c>
       <c r="E24" t="n">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F24" t="n">
         <v>4</v>
       </c>
       <c r="G24" t="n">
-        <v>164.2242940045646</v>
+        <v>168.2878187400502</v>
       </c>
       <c r="H24" t="n">
-        <v>391.6368421052632</v>
+        <v>395.8031914893617</v>
       </c>
       <c r="I24" t="n">
         <v>360</v>
@@ -8897,19 +8897,19 @@
         <v>74805</v>
       </c>
       <c r="E25" t="n">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>131.5842055163205</v>
+        <v>143.452020825728</v>
       </c>
       <c r="H25" t="n">
-        <v>390.151832460733</v>
+        <v>396.3776595744681</v>
       </c>
       <c r="I25" t="n">
-        <v>359</v>
+        <v>360.5</v>
       </c>
     </row>
     <row r="26">
@@ -9194,16 +9194,16 @@
         <v>71206</v>
       </c>
       <c r="E34" t="n">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>81.80332199863128</v>
+        <v>86.44747030628979</v>
       </c>
       <c r="H34" t="n">
-        <v>383.3513513513514</v>
+        <v>385.4347826086956</v>
       </c>
       <c r="I34" t="n">
         <v>372</v>
@@ -9293,19 +9293,19 @@
         <v>74926</v>
       </c>
       <c r="E37" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>245.5336134557088</v>
+        <v>240.7153613602697</v>
       </c>
       <c r="H37" t="n">
-        <v>425.9428571428571</v>
+        <v>423.5227272727273</v>
       </c>
       <c r="I37" t="n">
-        <v>325</v>
+        <v>325.5</v>
       </c>
     </row>
     <row r="38">
@@ -9326,16 +9326,16 @@
         <v>75112</v>
       </c>
       <c r="E38" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G38" t="n">
-        <v>317.4651104535074</v>
+        <v>309.3387451516551</v>
       </c>
       <c r="H38" t="n">
-        <v>482.9677419354838</v>
+        <v>476.8152866242038</v>
       </c>
       <c r="I38" t="n">
         <v>402</v>
@@ -9392,19 +9392,19 @@
         <v>74956</v>
       </c>
       <c r="E40" t="n">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="F40" t="n">
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>108.3509123776126</v>
+        <v>112.8372719575605</v>
       </c>
       <c r="H40" t="n">
-        <v>277.2230483271375</v>
+        <v>281.4075471698113</v>
       </c>
       <c r="I40" t="n">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="41">
@@ -9458,19 +9458,19 @@
         <v>72312</v>
       </c>
       <c r="E42" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F42" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G42" t="n">
-        <v>3789.194692995937</v>
+        <v>3657.18939670901</v>
       </c>
       <c r="H42" t="n">
-        <v>1995.583333333333</v>
+        <v>1842.076923076923</v>
       </c>
       <c r="I42" t="n">
-        <v>697</v>
+        <v>665</v>
       </c>
     </row>
     <row r="43">
@@ -9524,19 +9524,19 @@
         <v>74691</v>
       </c>
       <c r="E44" t="n">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F44" t="n">
         <v>5</v>
       </c>
       <c r="G44" t="n">
-        <v>158.5481758452075</v>
+        <v>161.317792085843</v>
       </c>
       <c r="H44" t="n">
-        <v>408.939226519337</v>
+        <v>411.2111111111111</v>
       </c>
       <c r="I44" t="n">
-        <v>378</v>
+        <v>378.5</v>
       </c>
     </row>
     <row r="45">
@@ -9722,19 +9722,19 @@
         <v>69142</v>
       </c>
       <c r="E50" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F50" t="n">
         <v>11</v>
       </c>
       <c r="G50" t="n">
-        <v>484.0356676316695</v>
+        <v>476.0496042769504</v>
       </c>
       <c r="H50" t="n">
-        <v>526.2213740458016</v>
+        <v>514.4402985074627</v>
       </c>
       <c r="I50" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="51">
@@ -9821,19 +9821,19 @@
         <v>74809</v>
       </c>
       <c r="E53" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F53" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G53" t="n">
-        <v>379.6282965642991</v>
+        <v>375.0804985021006</v>
       </c>
       <c r="H53" t="n">
-        <v>539.1666666666666</v>
+        <v>535.2877697841726</v>
       </c>
       <c r="I53" t="n">
-        <v>354.5</v>
+        <v>355</v>
       </c>
     </row>
     <row r="54">
@@ -9854,19 +9854,19 @@
         <v>68699</v>
       </c>
       <c r="E54" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>42.20928013523637</v>
+        <v>46.862181449816</v>
       </c>
       <c r="H54" t="n">
-        <v>347.7766497461929</v>
+        <v>349.5510204081633</v>
       </c>
       <c r="I54" t="n">
-        <v>344</v>
+        <v>344.5</v>
       </c>
     </row>
     <row r="55">
@@ -9920,19 +9920,19 @@
         <v>67780</v>
       </c>
       <c r="E56" t="n">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F56" t="n">
         <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>104.5473248930208</v>
+        <v>108.3900526106008</v>
       </c>
       <c r="H56" t="n">
-        <v>401.9761904761905</v>
+        <v>406.8192771084337</v>
       </c>
       <c r="I56" t="n">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="57">
@@ -9953,16 +9953,16 @@
         <v>75039</v>
       </c>
       <c r="E57" t="n">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>47.27652115729666</v>
+        <v>54.32676122248245</v>
       </c>
       <c r="H57" t="n">
-        <v>371.5422885572139</v>
+        <v>373.4</v>
       </c>
       <c r="I57" t="n">
         <v>372</v>
@@ -9986,19 +9986,19 @@
         <v>74875</v>
       </c>
       <c r="E58" t="n">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>136.4719505901947</v>
+        <v>138.7984203581202</v>
       </c>
       <c r="H58" t="n">
-        <v>323.7434782608696</v>
+        <v>325.1572052401747</v>
       </c>
       <c r="I58" t="n">
-        <v>311.5</v>
+        <v>312</v>
       </c>
     </row>
     <row r="59">
@@ -10019,16 +10019,16 @@
         <v>74901</v>
       </c>
       <c r="E59" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>35.37208925823384</v>
+        <v>43.43263855294165</v>
       </c>
       <c r="H59" t="n">
-        <v>372.535</v>
+        <v>374.4070351758794</v>
       </c>
       <c r="I59" t="n">
         <v>369</v>
@@ -10052,16 +10052,16 @@
         <v>61086</v>
       </c>
       <c r="E60" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F60" t="n">
         <v>1</v>
       </c>
       <c r="G60" t="n">
-        <v>131.3086737097403</v>
+        <v>133.750565379372</v>
       </c>
       <c r="H60" t="n">
-        <v>371.25</v>
+        <v>373.5276073619632</v>
       </c>
       <c r="I60" t="n">
         <v>329</v>
@@ -10118,16 +10118,16 @@
         <v>74711</v>
       </c>
       <c r="E62" t="n">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>28.8835747133455</v>
+        <v>36.62134682988943</v>
       </c>
       <c r="H62" t="n">
-        <v>314.1012658227848</v>
+        <v>315.4322033898305</v>
       </c>
       <c r="I62" t="n">
         <v>309</v>
@@ -10184,19 +10184,19 @@
         <v>93082</v>
       </c>
       <c r="E64" t="n">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>56.08284864630213</v>
+        <v>60.66522840924033</v>
       </c>
       <c r="H64" t="n">
-        <v>403.0478260869565</v>
+        <v>404.8078602620087</v>
       </c>
       <c r="I64" t="n">
-        <v>405.5</v>
+        <v>406</v>
       </c>
     </row>
     <row r="65">
@@ -10217,16 +10217,16 @@
         <v>22515</v>
       </c>
       <c r="E65" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F65" t="n">
         <v>2</v>
       </c>
       <c r="G65" t="n">
-        <v>260.7041066145176</v>
+        <v>310.1306370320448</v>
       </c>
       <c r="H65" t="n">
-        <v>458.5833333333333</v>
+        <v>468.3404255319149</v>
       </c>
       <c r="I65" t="n">
         <v>394</v>
@@ -10250,16 +10250,16 @@
         <v>70853</v>
       </c>
       <c r="E66" t="n">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F66" t="n">
         <v>3</v>
       </c>
       <c r="G66" t="n">
-        <v>119.6659502594983</v>
+        <v>121.2997934943841</v>
       </c>
       <c r="H66" t="n">
-        <v>386.3846153846154</v>
+        <v>388.5193370165746</v>
       </c>
       <c r="I66" t="n">
         <v>364</v>
@@ -10349,19 +10349,19 @@
         <v>54225</v>
       </c>
       <c r="E69" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F69" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G69" t="n">
-        <v>778.5223844738139</v>
+        <v>773.101480867737</v>
       </c>
       <c r="H69" t="n">
-        <v>642.6309523809524</v>
+        <v>635.0705882352942</v>
       </c>
       <c r="I69" t="n">
-        <v>396.5</v>
+        <v>397</v>
       </c>
     </row>
     <row r="70">
@@ -10382,19 +10382,19 @@
         <v>41858</v>
       </c>
       <c r="E70" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>78.05300140313237</v>
+        <v>85.51919179528628</v>
       </c>
       <c r="H70" t="n">
-        <v>387.4859813084112</v>
+        <v>391.1415094339623</v>
       </c>
       <c r="I70" t="n">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="71">
@@ -10448,19 +10448,19 @@
         <v>74992</v>
       </c>
       <c r="E72" t="n">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G72" t="n">
-        <v>81.53279570916249</v>
+        <v>98.53362661638681</v>
       </c>
       <c r="H72" t="n">
-        <v>410.8956043956044</v>
+        <v>415.4611111111111</v>
       </c>
       <c r="I72" t="n">
-        <v>407.5</v>
+        <v>408</v>
       </c>
     </row>
     <row r="73">
@@ -10481,19 +10481,19 @@
         <v>52248</v>
       </c>
       <c r="E73" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F73" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G73" t="n">
-        <v>628.0606939724934</v>
+        <v>620.8152448162034</v>
       </c>
       <c r="H73" t="n">
-        <v>653.632911392405</v>
+        <v>645.4625</v>
       </c>
       <c r="I73" t="n">
-        <v>417</v>
+        <v>437.5</v>
       </c>
     </row>
     <row r="74">

</xml_diff>